<commit_message>
Import official league results and scoring rules
</commit_message>
<xml_diff>
--- a/templates/wuri-league-demo-import.xlsx
+++ b/templates/wuri-league-demo-import.xlsx
@@ -430,7 +430,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>請勿修改欄位名稱；正式版型轉換器將在取得原始 Excel 後調整。</v>
+        <v>合法團體比分為 3–0、0–3、2–1、1–2；請勿修改欄位名稱。</v>
       </c>
     </row>
   </sheetData>
@@ -2322,10 +2322,10 @@
         <v>B-20261004-1</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
         <v>final</v>
@@ -2342,7 +2342,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="str">
         <v>final</v>

</xml_diff>